<commit_message>
Copy audit: identifier types read "Client SKU" / "Client barcode"
Closes the two rows left for a human in batch 2. Labels only; the keys
customer_sku and customer_barcode are unchanged. "customer POs" in the order
attachments hint stays as decided. Workbook rows marked; no human rows left.
sw.js CACHE_NAME -> v115.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsZ7iSWPcoTDJ2k5HWxMzx
</commit_message>
<xml_diff>
--- a/docs/COPY-AUDIT.xlsx
+++ b/docs/COPY-AUDIT.xlsx
@@ -15247,7 +15247,7 @@
         <v>html-text</v>
       </c>
       <c r="I512" t="str">
-        <v>human — "customer POs" on an order: the ship-to customer's PO or the client's? Left as is</v>
+        <v>kept — decided 2026-09-06: "customer POs" stays</v>
       </c>
     </row>
     <row r="513">
@@ -17509,7 +17509,7 @@
         <v>template-text</v>
       </c>
       <c r="I590" t="str">
-        <v>human — identifier type: whose SKU code? Left as is</v>
+        <v>applied: client SKU (label only, key customer_sku unchanged)</v>
       </c>
     </row>
     <row r="591">
@@ -18031,7 +18031,7 @@
         <v>option</v>
       </c>
       <c r="I608" t="str">
-        <v>human — identifier type, see "customer SKU"</v>
+        <v>applied: Client SKU (label only, key customer_sku unchanged)</v>
       </c>
     </row>
     <row r="609">
@@ -20583,7 +20583,7 @@
         <v>template-text</v>
       </c>
       <c r="I696" t="str">
-        <v>human — identifier type: is this the client's barcode or the ship-to customer's? Left as is</v>
+        <v>applied: client barcode (label only, key customer_barcode unchanged)</v>
       </c>
     </row>
     <row r="697">
@@ -20641,7 +20641,7 @@
         <v>option</v>
       </c>
       <c r="I698" t="str">
-        <v>human — identifier type, see "customer barcode"</v>
+        <v>applied: Client barcode (label only, key customer_barcode unchanged)</v>
       </c>
     </row>
     <row r="699">

</xml_diff>